<commit_message>
Inject category/featured metadata in adventure import
import-adventure-detail-page now appends per-adventure category and
featured (curated rank) rows to each page's Metadata block after
createMetadata, keyed by URL slug. This lands the values in <head> as
meta tags so the published query index carries them, powering the
Current Adventures category tabs and the homepage curated order.
Includes the rebuilt bundle and refreshed import reports.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-adventure-detail-page.report.xlsx
+++ b/tools/importer/reports/import-adventure-detail-page.report.xlsx
@@ -157,7 +157,7 @@
     <t>adventure-detail-page</t>
   </si>
   <si>
-    <t>2026-08-10T14:27:48.480Z</t>
+    <t>2026-08-10T20:21:16.087Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -172,7 +172,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-08-10T14:27:54.720Z</t>
+    <t>2026-08-10T20:21:21.528Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -187,7 +187,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:00.254Z</t>
+    <t>2026-08-10T20:21:26.748Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -202,7 +202,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:04.378Z</t>
+    <t>2026-08-10T20:21:32.942Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -217,7 +217,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:09.568Z</t>
+    <t>2026-08-10T20:21:37.968Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -232,7 +232,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:16.420Z</t>
+    <t>2026-08-10T20:21:43.237Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -247,7 +247,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:21.714Z</t>
+    <t>2026-08-10T20:21:48.012Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -262,7 +262,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:26.754Z</t>
+    <t>2026-08-10T20:21:53.361Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -277,7 +277,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:33.063Z</t>
+    <t>2026-08-10T20:21:59.430Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -292,7 +292,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:38.634Z</t>
+    <t>2026-08-10T20:22:07.007Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -307,7 +307,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:43.575Z</t>
+    <t>2026-08-10T20:22:12.269Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -322,7 +322,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:49.131Z</t>
+    <t>2026-08-10T20:22:18.085Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -337,7 +337,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-08-10T14:28:54.108Z</t>
+    <t>2026-08-10T20:22:22.552Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -352,7 +352,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-08-10T14:29:00.726Z</t>
+    <t>2026-08-10T20:22:27.370Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -367,7 +367,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-08-10T14:29:05.698Z</t>
+    <t>2026-08-10T20:22:32.138Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -382,7 +382,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-08-10T14:29:12.126Z</t>
+    <t>2026-08-10T20:22:37.673Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>

</xml_diff>